<commit_message>
Created the Data Provider Utility for Excel Data that is used in createdJobAPITest
Also Added FDLoginAPIExcelDataDrivenTest and
CreateJobAPIExcelDataDrivenTest in testng.xml
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/PhoenixTestData.xlsx
+++ b/src/test/resources/testData/PhoenixTestData.xlsx
@@ -1,22 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abhil\Downloads\Eclipse Workspace\PhoenixTestAutomationFramework\src\test\resources\testData\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{594E2FB3-D2C4-4A7D-BD78-F8AAB82A5927}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{16971C86-6B00-4FAA-A9B6-0B7AB5481250}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginTestData" sheetId="1" r:id="rId1"/>
     <sheet name="CreateJobTestData" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1:R27"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -26,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="49">
   <si>
     <t>username</t>
   </si>
@@ -44,13 +40,142 @@
   </si>
   <si>
     <t>iamsup</t>
+  </si>
+  <si>
+    <t>mst_service_location_id</t>
+  </si>
+  <si>
+    <t>mst_platform_id</t>
+  </si>
+  <si>
+    <t>mst_warrenty_status_id</t>
+  </si>
+  <si>
+    <t>mst_oem_id</t>
+  </si>
+  <si>
+    <t>customer__first_name</t>
+  </si>
+  <si>
+    <t>customer__last_name</t>
+  </si>
+  <si>
+    <t>customer__mobile_number</t>
+  </si>
+  <si>
+    <t>customer__mobile_number_alt</t>
+  </si>
+  <si>
+    <t>customer__email_id</t>
+  </si>
+  <si>
+    <t>customer__email_id_alt</t>
+  </si>
+  <si>
+    <t>customer_address__flat_number</t>
+  </si>
+  <si>
+    <t>customer_address__apartment_name</t>
+  </si>
+  <si>
+    <t>customer_address__street_name</t>
+  </si>
+  <si>
+    <t>customer_address__landmark</t>
+  </si>
+  <si>
+    <t>customer_address__area</t>
+  </si>
+  <si>
+    <t>customer_address__pincode</t>
+  </si>
+  <si>
+    <t>customer_address__country</t>
+  </si>
+  <si>
+    <t>customer_address__state</t>
+  </si>
+  <si>
+    <t>customer_product__dop</t>
+  </si>
+  <si>
+    <t>customer_product__serial_number</t>
+  </si>
+  <si>
+    <t>customer_product__imei1</t>
+  </si>
+  <si>
+    <t>customer_product__imei2</t>
+  </si>
+  <si>
+    <t>customer_product__popurl</t>
+  </si>
+  <si>
+    <t>customer_product__product_id</t>
+  </si>
+  <si>
+    <t>customer_product__mst_model_id</t>
+  </si>
+  <si>
+    <t>problems__id</t>
+  </si>
+  <si>
+    <t>problems__remark</t>
+  </si>
+  <si>
+    <t>Ruthie</t>
+  </si>
+  <si>
+    <t>Ryan</t>
+  </si>
+  <si>
+    <t>560-884-6559</t>
+  </si>
+  <si>
+    <t>Monserrat_VonRueden@hotmail.com</t>
+  </si>
+  <si>
+    <t>Test apartment</t>
+  </si>
+  <si>
+    <t>test street name</t>
+  </si>
+  <si>
+    <t>test landmark</t>
+  </si>
+  <si>
+    <t>test area</t>
+  </si>
+  <si>
+    <t>India</t>
+  </si>
+  <si>
+    <t>Madhya Pradesh</t>
+  </si>
+  <si>
+    <t>2026-04-30T20:00:00.000Z</t>
+  </si>
+  <si>
+    <t>handset overheats even after minimal usage.</t>
+  </si>
+  <si>
+    <t>14682142211476</t>
+  </si>
+  <si>
+    <t>14232142411476</t>
+  </si>
+  <si>
+    <t>14672142414486</t>
+  </si>
+  <si>
+    <t>14672242411789</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -58,16 +183,316 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri Light"/>
+      <family val="2"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -75,15 +500,207 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="42">
+    <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40% - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60% - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60% - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60% - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60% - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60% - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60% - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
+    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -411,9 +1028,438 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6EA6EE6-9721-4798-A590-01E03D47A522}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:AA5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="27" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="32.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="28.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="32.5546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="28.6640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="25.88671875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="24.6640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="24.44140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="23.21875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="30.109375" bestFit="1" customWidth="1"/>
+    <col min="21" max="22" width="22.77734375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="23.5546875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="27.21875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="30.109375" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="12" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="38.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="V1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="X1" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="Y1" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Z1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="AA1" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="A2" s="3">
+        <v>0</v>
+      </c>
+      <c r="B2" s="3">
+        <v>2</v>
+      </c>
+      <c r="C2" s="3">
+        <v>1</v>
+      </c>
+      <c r="D2" s="3">
+        <v>1</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3">
+        <v>10</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="P2" s="3">
+        <v>786543</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="W2" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="X2" s="3">
+        <v>1</v>
+      </c>
+      <c r="Y2" s="3">
+        <v>2</v>
+      </c>
+      <c r="Z2" s="3">
+        <v>6</v>
+      </c>
+      <c r="AA2" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="A3" s="3">
+        <v>0</v>
+      </c>
+      <c r="B3" s="3">
+        <v>2</v>
+      </c>
+      <c r="C3" s="3">
+        <v>1</v>
+      </c>
+      <c r="D3" s="3">
+        <v>1</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3">
+        <v>10</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="O3" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="P3" s="3">
+        <v>786543</v>
+      </c>
+      <c r="Q3" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="R3" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="S3" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="T3" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="U3" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="V3" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="W3" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="X3" s="3">
+        <v>1</v>
+      </c>
+      <c r="Y3" s="3">
+        <v>2</v>
+      </c>
+      <c r="Z3" s="3">
+        <v>6</v>
+      </c>
+      <c r="AA3" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="A4" s="3">
+        <v>0</v>
+      </c>
+      <c r="B4" s="3">
+        <v>2</v>
+      </c>
+      <c r="C4" s="3">
+        <v>1</v>
+      </c>
+      <c r="D4" s="3">
+        <v>1</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3">
+        <v>10</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="N4" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="O4" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="P4" s="3">
+        <v>786543</v>
+      </c>
+      <c r="Q4" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="R4" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="S4" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="T4" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="U4" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="V4" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="W4" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="X4" s="3">
+        <v>1</v>
+      </c>
+      <c r="Y4" s="3">
+        <v>2</v>
+      </c>
+      <c r="Z4" s="3">
+        <v>6</v>
+      </c>
+      <c r="AA4" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="A5" s="3">
+        <v>0</v>
+      </c>
+      <c r="B5" s="3">
+        <v>2</v>
+      </c>
+      <c r="C5" s="3">
+        <v>1</v>
+      </c>
+      <c r="D5" s="3">
+        <v>1</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3">
+        <v>10</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="N5" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="O5" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="P5" s="3">
+        <v>786543</v>
+      </c>
+      <c r="Q5" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="R5" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="S5" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="T5" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="U5" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="V5" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="W5" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="X5" s="3">
+        <v>1</v>
+      </c>
+      <c r="Y5" s="3">
+        <v>2</v>
+      </c>
+      <c r="Z5" s="3">
+        <v>6</v>
+      </c>
+      <c r="AA5" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>